<commit_message>
Align MO-433 confirm-accept page with Figma and drop locale churn.
Restore en/cy key order to main (confirmAccept only), match Figma copy/layout, and revert unrelated statement-view workbook noise.
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/19-producer-prns-prn-confirm-accept.xlsx
+++ b/translations/welsh-translations/xlsx/19-producer-prns-prn-confirm-accept.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="31">
   <si>
     <t>Translator notes</t>
   </si>
@@ -49,10 +49,13 @@
     <t>Confirmation page shown to producer before a PRN/PERN is accepted.</t>
   </si>
   <si>
-    <t>Confirm you want to accept this {{type}}</t>
+    <t>Accept this {{type}}</t>
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-112301</t>
   </si>
   <si>
     <t>prns.confirmAccept.heading</t>
@@ -550,7 +553,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
@@ -567,12 +570,12 @@
         <v>13</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>10</v>
@@ -581,7 +584,7 @@
         <v>11</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>13</v>
@@ -592,7 +595,7 @@
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>10</v>
@@ -601,7 +604,7 @@
         <v>11</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>13</v>
@@ -612,7 +615,7 @@
     </row>
     <row r="9" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>10</v>
@@ -621,7 +624,7 @@
         <v>11</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>13</v>
@@ -632,7 +635,7 @@
     </row>
     <row r="10" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>10</v>
@@ -641,7 +644,7 @@
         <v>11</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>13</v>
@@ -652,7 +655,7 @@
     </row>
     <row r="11" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>10</v>
@@ -661,7 +664,7 @@
         <v>11</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>13</v>
@@ -672,7 +675,7 @@
     </row>
     <row r="12" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>10</v>
@@ -681,7 +684,7 @@
         <v>11</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>13</v>
@@ -692,7 +695,7 @@
     </row>
     <row r="13" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>10</v>
@@ -701,7 +704,7 @@
         <v>11</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>13</v>
@@ -712,7 +715,7 @@
     </row>
     <row r="14" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>10</v>
@@ -721,7 +724,7 @@
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>13</v>
@@ -737,6 +740,9 @@
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="D3:F3"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="F6" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>